<commit_message>
chore(lem): re-save arai_tagyo input from Studio
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_arai_tagyo.xlsx
+++ b/docs/lem/files/xslope_arai_tagyo.xlsx
@@ -10169,7 +10169,7 @@
         <v>49</v>
       </c>
       <c r="D9" s="1">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>19</v>
@@ -10183,7 +10183,7 @@
         <v>48</v>
       </c>
       <c r="D10" s="1">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>17</v>
@@ -10198,7 +10198,7 @@
         <v>75</v>
       </c>
       <c r="D11" s="1">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>21</v>
@@ -12449,28 +12449,62 @@
       <c r="F9" s="3">
         <v>15.0</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
+      <c r="G9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J9" s="3">
+        <v>0.0</v>
+      </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="3"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
+      <c r="L9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="M9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="N9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="O9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="P9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="R9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="S9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="T9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="U9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="V9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="W9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="X9" s="3">
+        <v>0.0</v>
+      </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
@@ -13219,15 +13253,17 @@
         <v>46</v>
       </c>
       <c r="B2" s="3">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="D2" s="27" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="52" t="s">
-        <v>2</v>
+      <c r="A4" s="52" t="inlineStr">
+        <is>
+          <t>Profile Line #1</t>
+        </is>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="52" t="s">
@@ -13582,10 +13618,10 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
-        <v>0</v>
+        <v>-30.0</v>
       </c>
       <c r="B8" s="3">
-        <v>15</v>
+        <v>15.0</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
@@ -13626,10 +13662,10 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
-        <v>18</v>
+        <v>18.0</v>
       </c>
       <c r="B9" s="3">
-        <v>15</v>
+        <v>15.0</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
@@ -13670,10 +13706,10 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
-        <v>48</v>
+        <v>48.0</v>
       </c>
       <c r="B10" s="3">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
@@ -13714,10 +13750,10 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
-        <v>66</v>
+        <v>100.0</v>
       </c>
       <c r="B11" s="3">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -15868,17 +15904,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>33</v>
+        <v>33.0</v>
       </c>
       <c r="C3" s="3">
-        <v>55</v>
+        <v>55.0</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Intercept</t>
+          <t>Depth</t>
         </is>
       </c>
-      <c r="E3" s="3"/>
+      <c r="E3" s="3">
+        <v>12.2799812734</v>
+      </c>
       <c r="F3" s="3">
         <v>18</v>
       </c>
@@ -15898,10 +15936,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>35</v>
+        <v>35.0</v>
       </c>
       <c r="C4" s="3">
-        <v>55</v>
+        <v>55.0</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -15909,7 +15947,7 @@
         </is>
       </c>
       <c r="E4" s="3">
-        <v>0</v>
+        <v>0.0</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>

</xml_diff>